<commit_message>
Add builder commentary and a hand-entered approval to the dashboard
Each dashboard row gets a Builder commentary button that opens a window
with the variation's thread: every entry timestamped as it is added, with
who it is from and who entered it, saved to the log straight away. The
same window takes the approved value and date, typed from what the builder
approved; approving no longer copies in the schedule of rates' figure, and
the Approved total adds up only what was entered.

Entries are only ever added, each with an id, and the row is read again
before each dashboard write, so two people commenting at once keep both,
and a save from the form keeps what was added on the dashboard. The thread
also goes to the log as text in a new BuilderCommentary column.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0179JD8tKBuQw572uHNzHE2b
</commit_message>
<xml_diff>
--- a/registers/Variation Log.xlsx
+++ b/registers/Variation Log.xlsx
@@ -358,6 +358,11 @@
     <comment ref="AC4" authorId="1" shapeId="0">
       <text>
         <t>Date only. When it was approved, set on the project dashboard. Blank until then.</t>
+      </text>
+    </comment>
+    <comment ref="AD4" authorId="1" shapeId="0">
+      <text>
+        <t>Multiple lines of text, plain. The builder commentary thread from the project dashboard, as readable text, newest last. The app keeps its own copy in Payload.</t>
       </text>
     </comment>
   </commentList>
@@ -687,7 +692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC7"/>
+  <dimension ref="A1:AD7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -719,6 +724,7 @@
     <col width="16" customWidth="1" min="27" max="27"/>
     <col width="16" customWidth="1" min="28" max="28"/>
     <col width="16" customWidth="1" min="29" max="29"/>
+    <col width="40" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -881,6 +887,11 @@
           <t>ApprovedDate</t>
         </is>
       </c>
+      <c r="AD4" s="3" t="inlineStr">
+        <is>
+          <t>BuilderCommentary</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -1017,6 +1028,12 @@
       </c>
       <c r="AB5" s="4" t="n"/>
       <c r="AC5" s="4" t="n"/>
+      <c r="AD5" s="4" t="inlineStr">
+        <is>
+          <t>24 Oct 2026, 09:15 am — Spiros Laladakis, Built (entered by Adam Donnelly):
+Approved as submitted.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Print the PM's email on the letter, from the register's PmEmail column
The email in the letterhead and under the sign-off came from the office's
letterhead register. Both now come from a new PM email field in step 6,
filled from the project register's PmEmail column or typed in; the office
email stands in only when a project has none. One of the two is required,
in place of the office email.

The PM email goes to the log write and the filing flow as pmEmail, and
travels in the saved form, so the log, a reopened variation and the
variation file all keep it. It can be matched in Settings like the other
register columns. The registers, the Get projects Select step and the log
column list document it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0179JD8tKBuQw572uHNzHE2b
</commit_message>
<xml_diff>
--- a/registers/Variation Log.xlsx
+++ b/registers/Variation Log.xlsx
@@ -363,6 +363,11 @@
     <comment ref="AD4" authorId="1" shapeId="0">
       <text>
         <t>Multiple lines of text, plain. The builder commentary thread from the project dashboard, as readable text, newest last. The app keeps its own copy in Payload.</t>
+      </text>
+    </comment>
+    <comment ref="AE4" authorId="1" shapeId="0">
+      <text>
+        <t>Single line of text. The PM email the variation was issued with (from the project register's PmEmail, or typed on the cover sheet).</t>
       </text>
     </comment>
   </commentList>
@@ -692,7 +697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD7"/>
+  <dimension ref="A1:AE7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -725,6 +730,7 @@
     <col width="16" customWidth="1" min="28" max="28"/>
     <col width="16" customWidth="1" min="29" max="29"/>
     <col width="40" customWidth="1" min="30" max="30"/>
+    <col width="32" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -892,6 +898,11 @@
           <t>BuilderCommentary</t>
         </is>
       </c>
+      <c r="AE4" s="3" t="inlineStr">
+        <is>
+          <t>PmEmail</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -1032,6 +1043,11 @@
         <is>
           <t>24 Oct 2026, 09:15 am — Spiros Laladakis, Built (entered by Adam Donnelly):
 Approved as submitted.</t>
+        </is>
+      </c>
+      <c r="AE5" s="4" t="inlineStr">
+        <is>
+          <t>adam.donnelly@axisplumbing.com.au</t>
         </is>
       </c>
     </row>

</xml_diff>